<commit_message>
Entry for column names at table creation and bounce out of edit mode when enter is hit a second time.
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EC5534-59DD-42D5-B5CC-C208970652BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965BFEFD-9118-4C96-94C7-2373310A173B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$168</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1708,7 +1708,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1735,12 +1735,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1755,7 +1749,7 @@
       <patternFill patternType="lightGrid"/>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -1981,19 +1975,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -2012,7 +1993,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2119,38 +2100,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2159,7 +2140,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2170,12 +2151,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2497,6 +2472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O1078"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2554,7 +2530,7 @@
       <c r="N1" s="7"/>
       <c r="O1" s="8"/>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" hidden="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2583,7 +2559,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="75">
+    <row r="3" spans="1:15" ht="75" hidden="1">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2615,7 +2591,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" hidden="1">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2647,7 +2623,7 @@
       </c>
       <c r="L4"/>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" hidden="1">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2679,7 +2655,7 @@
       </c>
       <c r="L5"/>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" hidden="1">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2711,7 +2687,7 @@
       </c>
       <c r="L6"/>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" hidden="1">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2743,7 +2719,7 @@
       </c>
       <c r="L7"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" hidden="1">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2775,7 +2751,7 @@
       </c>
       <c r="L8"/>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" hidden="1">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2807,7 +2783,7 @@
       </c>
       <c r="L9"/>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" hidden="1">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2839,7 +2815,7 @@
       </c>
       <c r="L10"/>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" hidden="1">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2871,7 +2847,7 @@
       </c>
       <c r="L11"/>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" hidden="1">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2903,7 +2879,7 @@
       </c>
       <c r="L12"/>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" hidden="1">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2935,7 +2911,7 @@
       </c>
       <c r="L13"/>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" hidden="1">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2967,7 +2943,7 @@
       </c>
       <c r="L14"/>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" hidden="1">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2999,7 +2975,7 @@
       </c>
       <c r="L15"/>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" hidden="1">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3031,7 +3007,7 @@
       </c>
       <c r="L16"/>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" hidden="1">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3063,7 +3039,7 @@
       </c>
       <c r="L17"/>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" hidden="1">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3095,7 +3071,7 @@
       </c>
       <c r="L18"/>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" hidden="1">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3127,7 +3103,7 @@
       </c>
       <c r="L19"/>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" hidden="1">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3159,7 +3135,7 @@
       </c>
       <c r="L20"/>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" hidden="1">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3191,7 +3167,7 @@
       </c>
       <c r="L21"/>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" hidden="1">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3223,7 +3199,7 @@
       </c>
       <c r="L22"/>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" hidden="1">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3255,7 +3231,7 @@
       </c>
       <c r="L23"/>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:12" hidden="1">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3287,7 +3263,7 @@
       </c>
       <c r="L24"/>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" hidden="1">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3319,7 +3295,7 @@
       </c>
       <c r="L25"/>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" hidden="1">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3351,7 +3327,7 @@
       </c>
       <c r="L26"/>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" hidden="1">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -3380,7 +3356,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" hidden="1">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3412,7 +3388,7 @@
       </c>
       <c r="L28"/>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" hidden="1">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3444,7 +3420,7 @@
       </c>
       <c r="L29"/>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" hidden="1">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -3473,7 +3449,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" hidden="1">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3505,7 +3481,7 @@
       </c>
       <c r="L31"/>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" hidden="1">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -3534,7 +3510,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="45">
+    <row r="33" spans="1:12" ht="45" hidden="1">
       <c r="A33" s="4">
         <v>33</v>
       </c>
@@ -3566,7 +3542,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" hidden="1">
       <c r="A34" s="4">
         <v>34</v>
       </c>
@@ -3595,7 +3571,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" hidden="1">
       <c r="A35">
         <v>37</v>
       </c>
@@ -3627,7 +3603,7 @@
       </c>
       <c r="L35"/>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" hidden="1">
       <c r="A36" s="4">
         <v>38</v>
       </c>
@@ -3656,7 +3632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" hidden="1">
       <c r="A37" s="4">
         <v>40</v>
       </c>
@@ -3685,7 +3661,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" hidden="1">
       <c r="A38">
         <v>41</v>
       </c>
@@ -3715,7 +3691,7 @@
       </c>
       <c r="L38"/>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" hidden="1">
       <c r="A39">
         <v>42</v>
       </c>
@@ -3747,7 +3723,7 @@
       </c>
       <c r="L39"/>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" hidden="1">
       <c r="A40" s="4">
         <v>44</v>
       </c>
@@ -3779,7 +3755,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" hidden="1">
       <c r="A41" s="4">
         <v>45</v>
       </c>
@@ -3808,7 +3784,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" hidden="1">
       <c r="A42" s="4">
         <v>46</v>
       </c>
@@ -3837,7 +3813,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="120">
+    <row r="43" spans="1:12" ht="120" hidden="1">
       <c r="A43" s="4">
         <v>47</v>
       </c>
@@ -3869,7 +3845,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" hidden="1">
       <c r="A44">
         <v>48</v>
       </c>
@@ -3901,7 +3877,7 @@
       </c>
       <c r="L44"/>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" hidden="1">
       <c r="A45" s="4">
         <v>49</v>
       </c>
@@ -3930,7 +3906,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" hidden="1">
       <c r="A46" s="4">
         <v>50</v>
       </c>
@@ -3959,7 +3935,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" hidden="1">
       <c r="A47">
         <v>51</v>
       </c>
@@ -3991,7 +3967,7 @@
       </c>
       <c r="L47"/>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" hidden="1">
       <c r="A48" s="4">
         <v>57</v>
       </c>
@@ -4023,7 +3999,7 @@
       </c>
       <c r="L48"/>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" spans="1:12" hidden="1">
       <c r="A49" s="4">
         <v>58</v>
       </c>
@@ -4052,7 +4028,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:12" hidden="1">
       <c r="A50">
         <v>59</v>
       </c>
@@ -4084,7 +4060,7 @@
       </c>
       <c r="L50"/>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" spans="1:12" hidden="1">
       <c r="A51" s="4">
         <v>60</v>
       </c>
@@ -4113,7 +4089,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="1:12" hidden="1">
       <c r="A52" s="4">
         <v>62</v>
       </c>
@@ -4142,7 +4118,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:12">
+    <row r="53" spans="1:12" hidden="1">
       <c r="A53" s="4">
         <v>63</v>
       </c>
@@ -4172,7 +4148,7 @@
       </c>
       <c r="L53" s="6"/>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" spans="1:12" hidden="1">
       <c r="A54" s="4">
         <v>66</v>
       </c>
@@ -4204,7 +4180,7 @@
       </c>
       <c r="L54"/>
     </row>
-    <row r="55" spans="1:12">
+    <row r="55" spans="1:12" hidden="1">
       <c r="A55" s="4">
         <v>67</v>
       </c>
@@ -4233,7 +4209,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:12">
+    <row r="56" spans="1:12" hidden="1">
       <c r="A56" s="4">
         <v>69</v>
       </c>
@@ -4262,7 +4238,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="1:12" hidden="1">
       <c r="A57" s="4">
         <v>76</v>
       </c>
@@ -4291,7 +4267,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:12">
+    <row r="58" spans="1:12" hidden="1">
       <c r="A58" s="4">
         <v>76</v>
       </c>
@@ -4320,7 +4296,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="30">
+    <row r="59" spans="1:12" ht="30" hidden="1">
       <c r="A59" s="4">
         <v>82</v>
       </c>
@@ -4350,7 +4326,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:12">
+    <row r="60" spans="1:12" hidden="1">
       <c r="A60" s="4">
         <v>83</v>
       </c>
@@ -4383,7 +4359,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="61" spans="1:12">
+    <row r="61" spans="1:12" hidden="1">
       <c r="A61" s="4">
         <v>85</v>
       </c>
@@ -4413,7 +4389,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:12">
+    <row r="62" spans="1:12" hidden="1">
       <c r="A62" s="4">
         <v>32</v>
       </c>
@@ -4442,7 +4418,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:12">
+    <row r="63" spans="1:12" hidden="1">
       <c r="A63" s="4">
         <v>54</v>
       </c>
@@ -4468,7 +4444,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:12">
+    <row r="64" spans="1:12" hidden="1">
       <c r="A64" s="4">
         <v>61</v>
       </c>
@@ -4495,7 +4471,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" hidden="1">
       <c r="A65" s="4">
         <v>87</v>
       </c>
@@ -4522,7 +4498,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" hidden="1">
       <c r="A66" s="4">
         <v>89</v>
       </c>
@@ -4551,7 +4527,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" hidden="1">
       <c r="A67" s="4">
         <v>74</v>
       </c>
@@ -4578,7 +4554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" hidden="1">
       <c r="A68" s="4">
         <v>91</v>
       </c>
@@ -4604,7 +4580,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" hidden="1">
       <c r="A69" s="4">
         <v>92</v>
       </c>
@@ -4631,7 +4607,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30">
+    <row r="70" spans="1:12" ht="30" hidden="1">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -4660,7 +4636,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30">
+    <row r="71" spans="1:12" ht="30" hidden="1">
       <c r="A71" s="4">
         <v>78</v>
       </c>
@@ -4690,7 +4666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" hidden="1">
       <c r="A72" s="4">
         <v>93</v>
       </c>
@@ -4720,7 +4696,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" hidden="1">
       <c r="A73" s="4">
         <v>94</v>
       </c>
@@ -4750,7 +4726,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" hidden="1">
       <c r="A74" s="4">
         <v>98</v>
       </c>
@@ -4777,7 +4753,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" hidden="1">
       <c r="A75" s="4">
         <v>99</v>
       </c>
@@ -4809,7 +4785,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:12">
+    <row r="76" spans="1:12" hidden="1">
       <c r="A76" s="4">
         <v>90</v>
       </c>
@@ -4839,7 +4815,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="30">
+    <row r="77" spans="1:12" ht="30" hidden="1">
       <c r="A77" s="4">
         <v>95</v>
       </c>
@@ -4869,7 +4845,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="30">
+    <row r="78" spans="1:12" ht="30" hidden="1">
       <c r="A78" s="4">
         <v>96</v>
       </c>
@@ -4899,7 +4875,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30">
+    <row r="79" spans="1:12" ht="30" hidden="1">
       <c r="A79" s="4">
         <v>97</v>
       </c>
@@ -4932,7 +4908,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="80" spans="1:12">
+    <row r="80" spans="1:12" hidden="1">
       <c r="A80" s="4">
         <v>109</v>
       </c>
@@ -4961,7 +4937,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:12">
+    <row r="81" spans="1:12" hidden="1">
       <c r="A81" s="4">
         <v>110</v>
       </c>
@@ -4990,7 +4966,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="30">
+    <row r="82" spans="1:12" ht="30" hidden="1">
       <c r="A82" s="4">
         <v>111</v>
       </c>
@@ -5019,7 +4995,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="30">
+    <row r="83" spans="1:12" ht="30" hidden="1">
       <c r="A83" s="4">
         <v>125</v>
       </c>
@@ -5048,7 +5024,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:12">
+    <row r="84" spans="1:12" hidden="1">
       <c r="A84" s="4">
         <v>128</v>
       </c>
@@ -5077,7 +5053,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:12">
+    <row r="85" spans="1:12" hidden="1">
       <c r="A85" s="4">
         <v>129</v>
       </c>
@@ -5106,7 +5082,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:12">
+    <row r="86" spans="1:12" hidden="1">
       <c r="A86" s="4">
         <v>135</v>
       </c>
@@ -5135,7 +5111,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:12">
+    <row r="87" spans="1:12" hidden="1">
       <c r="A87" s="4">
         <v>133</v>
       </c>
@@ -5161,7 +5137,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:12">
+    <row r="88" spans="1:12" hidden="1">
       <c r="A88" s="4">
         <v>136</v>
       </c>
@@ -5190,7 +5166,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:12">
+    <row r="89" spans="1:12" hidden="1">
       <c r="A89" s="4">
         <v>134</v>
       </c>
@@ -5219,7 +5195,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:12">
+    <row r="90" spans="1:12" hidden="1">
       <c r="A90" s="4">
         <v>137</v>
       </c>
@@ -5248,7 +5224,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="30">
+    <row r="91" spans="1:12" ht="30" hidden="1">
       <c r="A91" s="4">
         <v>140</v>
       </c>
@@ -5277,7 +5253,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:12">
+    <row r="92" spans="1:12" hidden="1">
       <c r="A92" s="4">
         <v>141</v>
       </c>
@@ -5309,7 +5285,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="93" spans="1:12">
+    <row r="93" spans="1:12" hidden="1">
       <c r="A93" s="4">
         <v>35</v>
       </c>
@@ -5341,7 +5317,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:12" hidden="1">
       <c r="A94" s="4">
         <v>39</v>
       </c>
@@ -5370,7 +5346,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:12">
+    <row r="95" spans="1:12" hidden="1">
       <c r="A95" s="4">
         <v>43</v>
       </c>
@@ -5399,7 +5375,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:12">
+    <row r="96" spans="1:12" hidden="1">
       <c r="A96" s="4">
         <v>81</v>
       </c>
@@ -5431,7 +5407,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" hidden="1">
       <c r="A97" s="4">
         <v>120</v>
       </c>
@@ -5457,7 +5433,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" spans="1:11" hidden="1">
       <c r="A98" s="4">
         <v>101</v>
       </c>
@@ -5483,7 +5459,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:11">
+    <row r="99" spans="1:11" hidden="1">
       <c r="A99" s="4">
         <v>126</v>
       </c>
@@ -5512,7 +5488,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:11">
+    <row r="100" spans="1:11" hidden="1">
       <c r="A100" s="4">
         <v>131</v>
       </c>
@@ -5541,7 +5517,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:11">
+    <row r="101" spans="1:11" hidden="1">
       <c r="A101" s="4">
         <v>65</v>
       </c>
@@ -5568,7 +5544,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:11">
+    <row r="102" spans="1:11" hidden="1">
       <c r="A102" s="4">
         <v>119</v>
       </c>
@@ -5594,7 +5570,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:11">
+    <row r="103" spans="1:11" hidden="1">
       <c r="A103" s="4">
         <v>138</v>
       </c>
@@ -5623,7 +5599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:11">
+    <row r="104" spans="1:11" hidden="1">
       <c r="A104" s="4">
         <v>144</v>
       </c>
@@ -5649,7 +5625,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
+    <row r="105" spans="1:11" hidden="1">
       <c r="A105" s="4">
         <v>145</v>
       </c>
@@ -5672,7 +5648,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" hidden="1">
       <c r="A106" s="4">
         <v>118</v>
       </c>
@@ -5698,7 +5674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" spans="1:11" hidden="1">
       <c r="A107" s="4">
         <v>146</v>
       </c>
@@ -5724,7 +5700,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:11">
+    <row r="108" spans="1:11" hidden="1">
       <c r="A108" s="4">
         <v>73</v>
       </c>
@@ -5751,7 +5727,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:11">
+    <row r="109" spans="1:11" hidden="1">
       <c r="A109" s="4">
         <v>116</v>
       </c>
@@ -5777,7 +5753,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:11">
+    <row r="110" spans="1:11" hidden="1">
       <c r="A110" s="4">
         <v>145</v>
       </c>
@@ -5807,7 +5783,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:11">
+    <row r="111" spans="1:11" hidden="1">
       <c r="A111" s="4">
         <v>56</v>
       </c>
@@ -5834,7 +5810,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:11">
+    <row r="112" spans="1:11" hidden="1">
       <c r="A112" s="4">
         <v>104</v>
       </c>
@@ -5860,7 +5836,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:12" ht="30">
+    <row r="113" spans="1:12" ht="30" hidden="1">
       <c r="A113" s="4">
         <v>147</v>
       </c>
@@ -5889,7 +5865,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:12">
+    <row r="114" spans="1:12" hidden="1">
       <c r="A114" s="4">
         <v>146</v>
       </c>
@@ -5918,7 +5894,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="115" spans="1:12">
+    <row r="115" spans="1:12" hidden="1">
       <c r="A115" s="4">
         <v>150</v>
       </c>
@@ -5947,7 +5923,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="116" spans="1:12">
+    <row r="116" spans="1:12" hidden="1">
       <c r="A116" s="4">
         <v>151</v>
       </c>
@@ -6208,11 +6184,9 @@
       <c r="H124" s="13" t="s">
         <v>471</v>
       </c>
-      <c r="J124" s="38">
-        <v>2</v>
-      </c>
+      <c r="J124" s="38"/>
       <c r="K124" s="4" t="s">
-        <v>155</v>
+        <v>26</v>
       </c>
       <c r="L124" s="6" t="s">
         <v>480</v>
@@ -6413,7 +6387,7 @@
         <v>144</v>
       </c>
       <c r="J130" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>132</v>
@@ -10341,7 +10315,15 @@
       <c r="H1078" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L167" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L168" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="1.4.7"/>
+        <filter val="1.4.8"/>
+        <filter val="1.4.9"/>
+        <filter val="Roadmap"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L77">
       <sortCondition ref="J1:J77"/>
     </sortState>
@@ -15936,7 +15918,7 @@
       <c r="E7" s="43"/>
       <c r="F7" s="44"/>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" ht="15.75" thickBot="1">
       <c r="A8" s="47" t="s">
         <v>172</v>
       </c>
@@ -15954,12 +15936,12 @@
         <v>479</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" ht="15.75" thickBot="1">
       <c r="A9" s="47" t="s">
         <v>203</v>
       </c>
-      <c r="B9" s="61" t="s">
-        <v>256</v>
+      <c r="B9" s="60" t="s">
+        <v>475</v>
       </c>
       <c r="C9" s="51"/>
       <c r="D9" s="52" t="s">
@@ -15976,8 +15958,8 @@
       <c r="A10" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="B10" s="62" t="s">
-        <v>256</v>
+      <c r="B10" s="60" t="s">
+        <v>475</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>479</v>

</xml_diff>

<commit_message>
Display Post Details in Cell - WIP
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965BFEFD-9118-4C96-94C7-2373310A173B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{17D70A51-DD66-4820-AC52-3ED91A5F4110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="3" activeTab="8" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -21,13 +21,15 @@
     <sheet name="Number Data Shape" sheetId="4" r:id="rId6"/>
     <sheet name="Checkbox Data Shape" sheetId="7" r:id="rId7"/>
     <sheet name="Link Data Shape" sheetId="8" r:id="rId8"/>
-    <sheet name="Sheet3" sheetId="9" r:id="rId9"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId10"/>
+    <sheet name="Post Data Shape" sheetId="11" r:id="rId9"/>
+    <sheet name="Sheet3" sheetId="9" r:id="rId10"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$169</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1825" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1911" uniqueCount="508">
   <si>
     <t>Item</t>
   </si>
@@ -1664,6 +1666,78 @@
   </si>
   <si>
     <t>Make green cell border that shows the current cell go away when the block loses focus</t>
+  </si>
+  <si>
+    <t>1.4.10</t>
+  </si>
+  <si>
+    <t>Add WordPress content (post) content type</t>
+  </si>
+  <si>
+    <t>1.4.11</t>
+  </si>
+  <si>
+    <t>post</t>
+  </si>
+  <si>
+    <t>displayTitle</t>
+  </si>
+  <si>
+    <t>displayAuthor</t>
+  </si>
+  <si>
+    <t>displayExceprt</t>
+  </si>
+  <si>
+    <t>displayCoverImage</t>
+  </si>
+  <si>
+    <t>diplayPublishDate</t>
+  </si>
+  <si>
+    <t>diplayModifiedDate</t>
+  </si>
+  <si>
+    <t>displayShortContent</t>
+  </si>
+  <si>
+    <t>link | wide | narrow</t>
+  </si>
+  <si>
+    <t>linkLocation</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>displayTitleInCover</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>0=no display, &gt;1 = location priority</t>
+  </si>
+  <si>
+    <t>title | image</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>postId</t>
+  </si>
+  <si>
+    <t>postType</t>
+  </si>
+  <si>
+    <t>options{</t>
+  </si>
+  <si>
+    <t>Any post id</t>
+  </si>
+  <si>
+    <t>Any post type</t>
   </si>
 </sst>
 </file>
@@ -1993,7 +2067,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2078,43 +2152,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2143,7 +2180,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -2152,6 +2188,40 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5407,7 +5477,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="97" spans="1:11" hidden="1">
+    <row r="97" spans="1:12" hidden="1">
       <c r="A97" s="4">
         <v>120</v>
       </c>
@@ -5433,7 +5503,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:11" hidden="1">
+    <row r="98" spans="1:12" hidden="1">
       <c r="A98" s="4">
         <v>101</v>
       </c>
@@ -5459,7 +5529,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:11" hidden="1">
+    <row r="99" spans="1:12" hidden="1">
       <c r="A99" s="4">
         <v>126</v>
       </c>
@@ -5488,7 +5558,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:11" hidden="1">
+    <row r="100" spans="1:12" hidden="1">
       <c r="A100" s="4">
         <v>131</v>
       </c>
@@ -5517,7 +5587,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:11" hidden="1">
+    <row r="101" spans="1:12" hidden="1">
       <c r="A101" s="4">
         <v>65</v>
       </c>
@@ -5544,7 +5614,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:11" hidden="1">
+    <row r="102" spans="1:12" hidden="1">
       <c r="A102" s="4">
         <v>119</v>
       </c>
@@ -5570,7 +5640,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:11" hidden="1">
+    <row r="103" spans="1:12" hidden="1">
       <c r="A103" s="4">
         <v>138</v>
       </c>
@@ -5599,7 +5669,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:11" hidden="1">
+    <row r="104" spans="1:12" hidden="1">
       <c r="A104" s="4">
         <v>144</v>
       </c>
@@ -5625,7 +5695,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:11" hidden="1">
+    <row r="105" spans="1:12" hidden="1">
       <c r="A105" s="4">
         <v>145</v>
       </c>
@@ -5648,7 +5718,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:11" hidden="1">
+    <row r="106" spans="1:12" hidden="1">
       <c r="A106" s="4">
         <v>118</v>
       </c>
@@ -5674,7 +5744,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:11" hidden="1">
+    <row r="107" spans="1:12" hidden="1">
       <c r="A107" s="4">
         <v>146</v>
       </c>
@@ -5700,12 +5770,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:11" hidden="1">
+    <row r="108" spans="1:12">
       <c r="A108" s="4">
-        <v>73</v>
+        <v>161</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>212</v>
+        <v>485</v>
       </c>
       <c r="C108" s="15" t="s">
         <v>190</v>
@@ -5714,143 +5784,167 @@
         <v>17</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G108" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H108" s="13" t="s">
-        <v>330</v>
-      </c>
-      <c r="J108" s="5"/>
+        <v>484</v>
+      </c>
       <c r="K108" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:11" hidden="1">
+    <row r="109" spans="1:12">
       <c r="A109" s="4">
-        <v>116</v>
+        <v>159</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>228</v>
+        <v>482</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G109" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H109" s="13" t="s">
-        <v>330</v>
+        <v>486</v>
+      </c>
+      <c r="J109" s="4">
+        <v>1</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" hidden="1">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" ht="30">
       <c r="A110" s="4">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>384</v>
+        <v>460</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G110" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H110" s="13" t="s">
-        <v>332</v>
-      </c>
-      <c r="J110" s="5"/>
+        <v>486</v>
+      </c>
+      <c r="J110" s="4">
+        <v>4</v>
+      </c>
       <c r="K110" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="111" spans="1:11" hidden="1">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12">
       <c r="A111" s="4">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>388</v>
+        <v>239</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F111" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G111" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
-        <v>385</v>
-      </c>
-      <c r="J111" s="5"/>
+        <v>486</v>
+      </c>
+      <c r="J111" s="4">
+        <v>5</v>
+      </c>
       <c r="K111" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="112" spans="1:11" hidden="1">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" ht="45">
       <c r="A112" s="4">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>86</v>
+        <v>254</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G112" s="4" t="s">
+        <v>168</v>
+      </c>
       <c r="H112" s="13" t="s">
-        <v>385</v>
+        <v>486</v>
+      </c>
+      <c r="J112" s="5">
+        <v>6</v>
       </c>
       <c r="K112" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="113" spans="1:12" ht="30" hidden="1">
+        <v>256</v>
+      </c>
+      <c r="L112" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" ht="30">
       <c r="A113" s="4">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F113" s="4" t="s">
         <v>6</v>
@@ -5859,18 +5953,24 @@
         <v>7</v>
       </c>
       <c r="H113" s="13" t="s">
-        <v>385</v>
+        <v>486</v>
+      </c>
+      <c r="J113" s="5">
+        <v>7</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>26</v>
+        <v>256</v>
+      </c>
+      <c r="L113" s="4" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="114" spans="1:12" hidden="1">
       <c r="A114" s="4">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>190</v>
@@ -5879,45 +5979,40 @@
         <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G114" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H114" s="13" t="s">
-        <v>387</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="J114" s="5"/>
       <c r="K114" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="115" spans="1:12" hidden="1">
       <c r="A115" s="4">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>453</v>
+        <v>228</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G115" s="4" t="s">
-        <v>468</v>
-      </c>
       <c r="H115" s="13" t="s">
-        <v>390</v>
+        <v>330</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>26</v>
@@ -5925,10 +6020,10 @@
     </row>
     <row r="116" spans="1:12" hidden="1">
       <c r="A116" s="4">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>454</v>
+        <v>384</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>190</v>
@@ -5937,63 +6032,61 @@
         <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F116" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G116" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G116" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H116" s="13" t="s">
-        <v>390</v>
-      </c>
+        <v>332</v>
+      </c>
+      <c r="J116" s="5"/>
       <c r="K116" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:12">
+    <row r="117" spans="1:12" hidden="1">
       <c r="A117" s="4">
-        <v>149</v>
+        <v>56</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>254</v>
+        <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G117" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H117" s="13" t="s">
-        <v>466</v>
+        <v>385</v>
       </c>
       <c r="J117" s="5"/>
       <c r="K117" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="118" spans="1:12" ht="30">
+    <row r="118" spans="1:12" hidden="1">
       <c r="A118" s="4">
-        <v>152</v>
+        <v>104</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>459</v>
+        <v>216</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E118" s="4" t="s">
         <v>86</v>
@@ -6001,28 +6094,25 @@
       <c r="F118" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G118" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H118" s="13" t="s">
-        <v>466</v>
+        <v>385</v>
       </c>
       <c r="K118" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="119" spans="1:12" ht="30">
+    <row r="119" spans="1:12" ht="30" hidden="1">
       <c r="A119" s="4">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>461</v>
+        <v>386</v>
       </c>
       <c r="C119" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E119" s="4" t="s">
         <v>86</v>
@@ -6031,24 +6121,24 @@
         <v>6</v>
       </c>
       <c r="G119" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H119" s="13" t="s">
-        <v>466</v>
+        <v>385</v>
       </c>
       <c r="K119" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="120" spans="1:12" ht="45">
+    <row r="120" spans="1:12" hidden="1">
       <c r="A120" s="4">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>465</v>
+        <v>214</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>17</v>
@@ -6057,156 +6147,150 @@
         <v>55</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G120" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H120" s="13" t="s">
-        <v>466</v>
+        <v>387</v>
       </c>
       <c r="K120" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L120" s="4" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="121" spans="1:12" ht="30">
+    </row>
+    <row r="121" spans="1:12" hidden="1">
       <c r="A121" s="4">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>470</v>
+        <v>453</v>
       </c>
       <c r="C121" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G121" s="4" t="s">
-        <v>168</v>
+        <v>468</v>
       </c>
       <c r="H121" s="13" t="s">
-        <v>469</v>
+        <v>390</v>
       </c>
       <c r="K121" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="122" spans="1:12" ht="30">
+    <row r="122" spans="1:12" hidden="1">
       <c r="A122" s="4">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>483</v>
+        <v>454</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E122" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G122" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H122" s="13" t="s">
-        <v>469</v>
+        <v>390</v>
       </c>
       <c r="K122" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="123" spans="1:12">
+    <row r="123" spans="1:12" hidden="1">
       <c r="A123" s="4">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>217</v>
+        <v>392</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>55</v>
+        <v>254</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G123" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H123" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J123" s="38">
-        <v>1</v>
-      </c>
+        <v>466</v>
+      </c>
+      <c r="J123" s="5"/>
       <c r="K123" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="L123" s="4" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" ht="30" hidden="1">
       <c r="A124" s="4">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>481</v>
+        <v>459</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H124" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J124" s="38"/>
+        <v>466</v>
+      </c>
       <c r="K124" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L124" s="6" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12">
+    </row>
+    <row r="125" spans="1:12" ht="30" hidden="1">
       <c r="A125" s="4">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>6</v>
@@ -6215,30 +6299,27 @@
         <v>11</v>
       </c>
       <c r="H125" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J125" s="38">
-        <v>3</v>
+        <v>466</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="126" spans="1:12" ht="30">
+    <row r="126" spans="1:12" ht="45" hidden="1">
       <c r="A126" s="4">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="C126" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
         <v>6</v>
@@ -6247,21 +6328,21 @@
         <v>11</v>
       </c>
       <c r="H126" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J126" s="38">
-        <v>4</v>
+        <v>466</v>
       </c>
       <c r="K126" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="127" spans="1:12">
+        <v>26</v>
+      </c>
+      <c r="L126" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" ht="30" hidden="1">
       <c r="A127" s="4">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>239</v>
+        <v>470</v>
       </c>
       <c r="C127" s="15" t="s">
         <v>189</v>
@@ -6270,176 +6351,152 @@
         <v>39</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G127" s="4" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="H127" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J127" s="38">
-        <v>5</v>
+        <v>469</v>
       </c>
       <c r="K127" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="128" spans="1:12" ht="45">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" ht="30" hidden="1">
       <c r="A128" s="4">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>253</v>
+        <v>483</v>
       </c>
       <c r="C128" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>39</v>
+        <v>307</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>254</v>
+        <v>86</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G128" s="4" t="s">
-        <v>168</v>
+        <v>11</v>
       </c>
       <c r="H128" s="13" t="s">
-        <v>471</v>
-      </c>
-      <c r="J128" s="39">
-        <v>6</v>
+        <v>469</v>
       </c>
       <c r="K128" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L128" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="129" spans="1:12" ht="30">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" hidden="1">
       <c r="A129" s="4">
-        <v>148</v>
+        <v>105</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>389</v>
+        <v>217</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="E129" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F129" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G129" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H129" s="13" t="s">
         <v>471</v>
       </c>
-      <c r="J129" s="39">
-        <v>7</v>
-      </c>
       <c r="K129" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
       <c r="L129" s="4" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="130" spans="1:12">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" hidden="1">
       <c r="A130" s="4">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G130" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H130" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I130" s="5">
-        <v>144</v>
-      </c>
-      <c r="J130" s="4">
-        <v>20</v>
+        <v>471</v>
       </c>
       <c r="K130" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12">
+        <v>26</v>
+      </c>
+      <c r="L130" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" hidden="1">
       <c r="A131" s="4">
-        <v>77</v>
+        <v>156</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>141</v>
+        <v>463</v>
       </c>
       <c r="C131" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G131" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H131" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I131" s="5">
-        <v>80</v>
-      </c>
-      <c r="J131" s="5">
-        <v>20</v>
+        <v>471</v>
       </c>
       <c r="K131" s="4" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
     </row>
     <row r="132" spans="1:12">
       <c r="A132" s="4">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="C132" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F132" s="4" t="s">
         <v>25</v>
@@ -6447,6 +6504,9 @@
       <c r="H132" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I132" s="5">
+        <v>80</v>
+      </c>
       <c r="J132" s="5">
         <v>20</v>
       </c>
@@ -6456,27 +6516,27 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C133" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J133" s="4">
+      <c r="J133" s="5">
         <v>20</v>
       </c>
       <c r="K133" s="4" t="s">
@@ -6485,13 +6545,13 @@
     </row>
     <row r="134" spans="1:12">
       <c r="A134" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C134" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D134" s="4" t="s">
         <v>18</v>
@@ -6500,10 +6560,7 @@
         <v>55</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G134" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
@@ -6514,31 +6571,28 @@
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L134" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="135" spans="1:12">
       <c r="A135" s="4">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>331</v>
+        <v>244</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
@@ -6549,13 +6603,16 @@
       <c r="K135" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L135" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="136" spans="1:12">
       <c r="A136" s="4">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>149</v>
+        <v>331</v>
       </c>
       <c r="C136" s="15" t="s">
         <v>189</v>
@@ -6564,19 +6621,19 @@
         <v>17</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G136" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J136" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>132</v>
@@ -6584,13 +6641,13 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C137" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>17</v>
@@ -6599,7 +6656,10 @@
         <v>55</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G137" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H137" s="13" t="s">
         <v>132</v>
@@ -6613,24 +6673,21 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C138" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G138" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H138" s="13" t="s">
@@ -6645,21 +6702,24 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C139" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E139" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F139" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G139" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H139" s="13" t="s">
@@ -6672,12 +6732,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:12" ht="30">
+    <row r="140" spans="1:12">
       <c r="A140" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>190</v>
@@ -6701,12 +6761,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="141" spans="1:12">
+    <row r="141" spans="1:12" ht="30">
       <c r="A141" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C141" s="15" t="s">
         <v>190</v>
@@ -6732,10 +6792,10 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C142" s="15" t="s">
         <v>190</v>
@@ -6744,19 +6804,16 @@
         <v>17</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I142" s="5">
-        <v>139</v>
-      </c>
-      <c r="J142" s="5">
-        <v>40</v>
+      <c r="J142" s="4">
+        <v>30</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>132</v>
@@ -6764,10 +6821,10 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>190</v>
@@ -6776,18 +6833,18 @@
         <v>17</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H143" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I143" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J143" s="4">
+      <c r="I143" s="5">
+        <v>139</v>
+      </c>
+      <c r="J143" s="5">
         <v>40</v>
       </c>
       <c r="K143" s="4" t="s">
@@ -6796,29 +6853,29 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C144" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F144" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G144" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H144" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I144" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J144" s="4">
         <v>40</v>
       </c>
@@ -6828,10 +6885,10 @@
     </row>
     <row r="145" spans="1:12">
       <c r="A145" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>189</v>
@@ -6858,12 +6915,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="146" spans="1:12" ht="30">
+    <row r="146" spans="1:12">
       <c r="A146" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>189</v>
@@ -6872,10 +6929,10 @@
         <v>17</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G146" s="4" t="s">
         <v>11</v>
@@ -6884,7 +6941,7 @@
         <v>132</v>
       </c>
       <c r="J146" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K146" s="4" t="s">
         <v>132</v>
@@ -6892,39 +6949,42 @@
     </row>
     <row r="147" spans="1:12" ht="30">
       <c r="A147" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C147" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F147" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G147" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H147" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J147" s="5">
+      <c r="J147" s="4">
         <v>50</v>
       </c>
       <c r="K147" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="148" spans="1:12">
+    <row r="148" spans="1:12" ht="30">
       <c r="A148" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>190</v>
@@ -6950,10 +7010,10 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C149" s="15" t="s">
         <v>190</v>
@@ -6962,15 +7022,15 @@
         <v>17</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H149" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J149" s="4">
+      <c r="J149" s="5">
         <v>50</v>
       </c>
       <c r="K149" s="4" t="s">
@@ -6979,10 +7039,10 @@
     </row>
     <row r="150" spans="1:12">
       <c r="A150" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C150" s="15" t="s">
         <v>190</v>
@@ -6994,7 +7054,7 @@
         <v>55</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H150" s="13" t="s">
         <v>132</v>
@@ -7008,22 +7068,22 @@
     </row>
     <row r="151" spans="1:12">
       <c r="A151" s="4">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C151" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E151" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H151" s="13" t="s">
         <v>132</v>
@@ -7037,13 +7097,13 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="4">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="C152" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>18</v>
@@ -7052,10 +7112,7 @@
         <v>55</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G152" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H152" s="13" t="s">
         <v>132</v>
@@ -7066,48 +7123,48 @@
       <c r="K152" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L152" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="153" spans="1:12" ht="30">
+    </row>
+    <row r="153" spans="1:12">
       <c r="A153" s="4">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>322</v>
+        <v>247</v>
       </c>
       <c r="C153" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E153" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G153" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H153" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I153" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J153" s="4">
         <v>50</v>
       </c>
       <c r="K153" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="154" spans="1:12">
+      <c r="L153" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12" ht="30">
       <c r="A154" s="4">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>218</v>
+        <v>322</v>
       </c>
       <c r="C154" s="15" t="s">
         <v>190</v>
@@ -7119,13 +7176,16 @@
         <v>55</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H154" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I154" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J154" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K154" s="4" t="s">
         <v>132</v>
@@ -7133,19 +7193,19 @@
     </row>
     <row r="155" spans="1:12">
       <c r="A155" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C155" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F155" s="4" t="s">
         <v>25</v>
@@ -7153,8 +7213,8 @@
       <c r="H155" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J155" s="5">
-        <v>80</v>
+      <c r="J155" s="4">
+        <v>60</v>
       </c>
       <c r="K155" s="4" t="s">
         <v>132</v>
@@ -7162,10 +7222,10 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C156" s="15" t="s">
         <v>189</v>
@@ -7191,10 +7251,10 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C157" s="15" t="s">
         <v>189</v>
@@ -7203,12 +7263,15 @@
         <v>17</v>
       </c>
       <c r="E157" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H157" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J157" s="4">
+      <c r="J157" s="5">
         <v>80</v>
       </c>
       <c r="K157" s="4" t="s">
@@ -7217,42 +7280,36 @@
     </row>
     <row r="158" spans="1:12">
       <c r="A158" s="4">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>29</v>
+        <v>219</v>
       </c>
       <c r="C158" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D158" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F158" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G158" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H158" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J158" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K158" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="159" spans="1:12" ht="30">
+    <row r="159" spans="1:12">
       <c r="A159" s="4">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C159" s="15" t="s">
         <v>189</v>
@@ -7261,7 +7318,7 @@
         <v>18</v>
       </c>
       <c r="E159" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>6</v>
@@ -7278,16 +7335,13 @@
       <c r="K159" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L159" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12">
+    </row>
+    <row r="160" spans="1:12" ht="30">
       <c r="A160" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C160" s="15" t="s">
         <v>189</v>
@@ -7296,13 +7350,13 @@
         <v>18</v>
       </c>
       <c r="E160" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F160" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G160" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H160" s="13" t="s">
         <v>132</v>
@@ -7313,13 +7367,16 @@
       <c r="K160" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L160" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="161" spans="1:12">
       <c r="A161" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C161" s="15" t="s">
         <v>189</v>
@@ -7328,13 +7385,13 @@
         <v>18</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G161" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H161" s="13" t="s">
         <v>132</v>
@@ -7346,24 +7403,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="162" spans="1:12" ht="30">
+    <row r="162" spans="1:12">
       <c r="A162" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C162" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D162" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E162" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F162" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G162" s="4" t="s">
         <v>24</v>
@@ -7380,10 +7437,10 @@
     </row>
     <row r="163" spans="1:12" ht="30">
       <c r="A163" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C163" s="15" t="s">
         <v>189</v>
@@ -7410,27 +7467,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="164" spans="1:12">
+    <row r="164" spans="1:12" ht="30">
       <c r="A164" s="4">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C164" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D164" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F164" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G164" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H164" s="13" t="s">
         <v>132</v>
@@ -7442,27 +7499,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="165" spans="1:12" ht="30">
+    <row r="165" spans="1:12">
       <c r="A165" s="4">
-        <v>139</v>
+        <v>88</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="C165" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D165" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E165" s="4" t="s">
-        <v>310</v>
+        <v>131</v>
       </c>
       <c r="F165" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G165" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H165" s="13" t="s">
         <v>132</v>
@@ -7473,31 +7530,28 @@
       <c r="K165" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L165" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="166" spans="1:12" ht="45">
+    </row>
+    <row r="166" spans="1:12" ht="30">
       <c r="A166" s="4">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="C166" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D166" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E166" s="4" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="F166" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G166" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H166" s="13" t="s">
         <v>132</v>
@@ -7509,24 +7563,24 @@
         <v>132</v>
       </c>
       <c r="L166" s="4" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
     </row>
     <row r="167" spans="1:12" ht="45">
       <c r="A167" s="4">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>462</v>
+        <v>319</v>
       </c>
       <c r="C167" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D167" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E167" s="4" t="s">
-        <v>86</v>
+        <v>320</v>
       </c>
       <c r="F167" s="4" t="s">
         <v>6</v>
@@ -7543,22 +7597,25 @@
       <c r="K167" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="168" spans="1:12" ht="30">
+      <c r="L167" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" ht="45">
       <c r="A168" s="4">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C168" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D168" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F168" s="4" t="s">
         <v>6</v>
@@ -7576,8 +7633,37 @@
         <v>132</v>
       </c>
     </row>
-    <row r="169" spans="1:12">
-      <c r="H169" s="13"/>
+    <row r="169" spans="1:12" ht="30">
+      <c r="A169" s="4">
+        <v>157</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="C169" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D169" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E169" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F169" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G169" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H169" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J169" s="4">
+        <v>99</v>
+      </c>
+      <c r="K169" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="170" spans="1:12">
       <c r="H170" s="13"/>
@@ -7621,7 +7707,7 @@
     <row r="183" spans="1:8">
       <c r="A183" s="9">
         <f>MAX(A1:A182)</f>
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B183" s="9" t="s">
         <v>95</v>
@@ -10315,12 +10401,11 @@
       <c r="H1078" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L168" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L169" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.4.7"/>
-        <filter val="1.4.8"/>
-        <filter val="1.4.9"/>
+        <filter val="1.4.10"/>
+        <filter val="1.4.11"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>
@@ -10328,10 +10413,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L168">
-    <sortCondition ref="H2:H168"/>
-    <sortCondition ref="J2:J168"/>
-    <sortCondition ref="A2:A168"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L169">
+    <sortCondition ref="H2:H169"/>
+    <sortCondition ref="J2:J169"/>
+    <sortCondition ref="A2:A169"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10339,6 +10424,147 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AB0EEF-943E-4A80-BEA9-7E9C713A7508}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="4" width="22.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="23.25">
+      <c r="A1" s="26" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="27" t="s">
+        <v>426</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>427</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>428</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="30">
+      <c r="A4" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>430</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30">
+      <c r="A5" s="29" t="s">
+        <v>431</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>433</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="30">
+      <c r="A6" s="29" t="s">
+        <v>434</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>435</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="45">
+      <c r="A7" s="29" t="s">
+        <v>436</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>437</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="29" t="s">
+        <v>400</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>438</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30">
+      <c r="A9" s="29" t="s">
+        <v>439</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>440</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="30"/>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="31" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="31" t="s">
+        <v>444</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
   <dimension ref="B9:T43"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -10891,43 +11117,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="50" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="19"/>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="49" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="34"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="49"/>
+      <c r="F1" s="47" t="s">
         <v>197</v>
       </c>
-      <c r="G1" s="32" t="s">
+      <c r="G1" s="47" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="47" t="s">
         <v>175</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="I1" s="47" t="s">
         <v>177</v>
       </c>
-      <c r="J1" s="34" t="s">
+      <c r="J1" s="49" t="s">
         <v>187</v>
       </c>
-      <c r="K1" s="34"/>
-      <c r="L1" s="32" t="s">
+      <c r="K1" s="49"/>
+      <c r="L1" s="47" t="s">
         <v>179</v>
       </c>
-      <c r="M1" s="32" t="s">
+      <c r="M1" s="47" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:45" ht="30.75" customHeight="1">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
+      <c r="A2" s="51"/>
+      <c r="B2" s="51"/>
       <c r="C2" s="20" t="s">
         <v>16</v>
       </c>
@@ -10937,18 +11163,18 @@
       <c r="E2" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
       <c r="J2" s="18" t="s">
         <v>185</v>
       </c>
       <c r="K2" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -11228,7 +11454,7 @@
     </row>
     <row r="7" spans="1:45" ht="60">
       <c r="A7" s="4" t="s">
-        <v>199</v>
+        <v>155</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>7</v>
@@ -11301,12 +11527,14 @@
     </row>
     <row r="8" spans="1:45">
       <c r="A8" s="4" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="15"/>
+      <c r="C8" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="D8" s="13" t="s">
         <v>390</v>
       </c>
@@ -11470,7 +11698,7 @@
     </row>
     <row r="11" spans="1:45">
       <c r="A11" s="4" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>11</v>
@@ -15873,143 +16101,143 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="24" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="44" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="44" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" thickBot="1"/>
     <row r="6" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="32" t="s">
         <v>474</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="52" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="52" t="s">
         <v>203</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="55" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="33" t="s">
         <v>473</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="44"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="56"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="34" t="s">
         <v>172</v>
       </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="60" t="s">
+      <c r="B8" s="36"/>
+      <c r="C8" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="D8" s="60" t="s">
+      <c r="D8" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="E8" s="60" t="s">
+      <c r="E8" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="F8" s="50" t="s">
+      <c r="F8" s="37" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="34" t="s">
         <v>203</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="C9" s="51"/>
-      <c r="D9" s="52" t="s">
+      <c r="C9" s="38"/>
+      <c r="D9" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="E9" s="52" t="s">
+      <c r="E9" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="F9" s="53" t="s">
+      <c r="F9" s="40" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="34" t="s">
         <v>174</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="C10" s="52" t="s">
+      <c r="C10" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="D10" s="51"/>
-      <c r="E10" s="52" t="s">
+      <c r="D10" s="38"/>
+      <c r="E10" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="F10" s="53" t="s">
+      <c r="F10" s="40" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="47" t="s">
+      <c r="A11" s="34" t="s">
         <v>206</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="45" t="s">
         <v>475</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="39" t="s">
         <v>479</v>
       </c>
-      <c r="E11" s="51"/>
-      <c r="F11" s="53" t="s">
+      <c r="E11" s="38"/>
+      <c r="F11" s="40" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A12" s="48" t="s">
+      <c r="A12" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="C12" s="55" t="s">
+      <c r="C12" s="42" t="s">
         <v>479</v>
       </c>
-      <c r="D12" s="55" t="s">
+      <c r="D12" s="42" t="s">
         <v>479</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="42" t="s">
         <v>479</v>
       </c>
-      <c r="F12" s="56"/>
+      <c r="F12" s="43"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="57"/>
+      <c r="A15" s="24"/>
     </row>
     <row r="24" spans="9:9">
       <c r="I24" s="6"/>
@@ -16042,13 +16270,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="57" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
       <c r="G2" s="21" t="s">
         <v>447</v>
       </c>
@@ -16195,13 +16423,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="57" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
       <c r="G2" s="21" t="s">
         <v>447</v>
       </c>
@@ -16390,13 +16618,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="57" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
       <c r="G2" s="21" t="s">
         <v>447</v>
       </c>
@@ -16585,13 +16813,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="57" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
       <c r="G2" s="21" t="s">
         <v>447</v>
       </c>
@@ -16868,142 +17096,355 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AB0EEF-943E-4A80-BEA9-7E9C713A7508}">
-  <dimension ref="A1:D16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF1C5E1A-770F-4373-A00C-9AD1A6999945}">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="B2:K37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="3" max="4" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="2" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" customWidth="1"/>
+    <col min="8" max="8" width="24.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" customWidth="1"/>
+    <col min="10" max="10" width="41.28515625" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.25">
-      <c r="A1" s="26" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="27" t="s">
-        <v>426</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>427</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>428</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="30">
-      <c r="A4" s="29" t="s">
-        <v>398</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>430</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30">
-      <c r="A5" s="29" t="s">
-        <v>431</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>432</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>433</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30">
-      <c r="A6" s="29" t="s">
-        <v>434</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>435</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="45">
-      <c r="A7" s="29" t="s">
-        <v>436</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>437</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="29" t="s">
+    <row r="2" spans="2:11">
+      <c r="B2" s="57" t="s">
+        <v>276</v>
+      </c>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="21" t="s">
+        <v>447</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="J2" s="21" t="s">
+        <v>289</v>
+      </c>
+      <c r="K2" s="21" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11">
+      <c r="B3" s="24" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11">
+      <c r="B4" t="s">
+        <v>264</v>
+      </c>
+      <c r="H4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11">
+      <c r="C5" t="s">
+        <v>265</v>
+      </c>
+      <c r="H5" t="s">
+        <v>266</v>
+      </c>
+      <c r="I5" t="s">
+        <v>395</v>
+      </c>
+      <c r="J5" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11">
+      <c r="C6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11">
+      <c r="D7" t="s">
+        <v>268</v>
+      </c>
+      <c r="H7" t="s">
+        <v>277</v>
+      </c>
+      <c r="I7" t="s">
+        <v>396</v>
+      </c>
+      <c r="J7" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11">
+      <c r="D8" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11">
+      <c r="F9" t="s">
+        <v>488</v>
+      </c>
+      <c r="G9" t="s">
+        <v>499</v>
+      </c>
+      <c r="I9" s="58">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11">
+      <c r="F10" t="s">
+        <v>491</v>
+      </c>
+      <c r="G10" t="s">
+        <v>499</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11">
+      <c r="F11" t="s">
+        <v>490</v>
+      </c>
+      <c r="G11" t="s">
+        <v>499</v>
+      </c>
+      <c r="I11" s="12">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11">
+      <c r="F12" t="s">
+        <v>489</v>
+      </c>
+      <c r="G12" t="s">
+        <v>499</v>
+      </c>
+      <c r="I12" s="12">
+        <v>0</v>
+      </c>
+      <c r="J12" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11">
+      <c r="F13" t="s">
+        <v>494</v>
+      </c>
+      <c r="G13" t="s">
+        <v>499</v>
+      </c>
+      <c r="I13" s="12">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11">
+      <c r="F14" t="s">
+        <v>492</v>
+      </c>
+      <c r="G14" t="s">
+        <v>499</v>
+      </c>
+      <c r="I14" s="12">
+        <v>0</v>
+      </c>
+      <c r="J14" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11">
+      <c r="F15" t="s">
+        <v>493</v>
+      </c>
+      <c r="G15" t="s">
+        <v>499</v>
+      </c>
+      <c r="I15" s="12">
+        <v>0</v>
+      </c>
+      <c r="J15" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11">
+      <c r="F16" t="s">
+        <v>498</v>
+      </c>
+      <c r="G16" t="s">
+        <v>448</v>
+      </c>
+      <c r="I16" s="22" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11">
+      <c r="F17" t="s">
+        <v>496</v>
+      </c>
+      <c r="G17" t="s">
+        <v>497</v>
+      </c>
+      <c r="I17" t="s">
+        <v>502</v>
+      </c>
+      <c r="J17" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11">
+      <c r="D18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11">
+      <c r="C19" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11">
+      <c r="B20" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11">
+      <c r="B22" s="24" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11">
+      <c r="B23" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11">
+      <c r="C24" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11">
+      <c r="D25" t="s">
+        <v>503</v>
+      </c>
+      <c r="G25" t="s">
+        <v>499</v>
+      </c>
+      <c r="J25" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11">
+      <c r="D26" t="s">
+        <v>504</v>
+      </c>
+      <c r="G26" t="s">
+        <v>396</v>
+      </c>
+      <c r="J26" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11">
+      <c r="C27" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11">
+      <c r="C28" t="s">
+        <v>419</v>
+      </c>
+      <c r="K28" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11">
+      <c r="D29" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11">
+      <c r="C30" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11">
+      <c r="C31" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11">
+      <c r="D32" t="s">
+        <v>445</v>
+      </c>
+      <c r="G32" t="s">
+        <v>448</v>
+      </c>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="J32" t="s">
+        <v>291</v>
+      </c>
+      <c r="K32" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11">
+      <c r="C33" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11">
+      <c r="C34" t="s">
+        <v>421</v>
+      </c>
+      <c r="K34" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11">
+      <c r="C35" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11">
+      <c r="C36" t="s">
         <v>400</v>
       </c>
-      <c r="B8" s="28" t="s">
-        <v>438</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="30">
-      <c r="A9" s="29" t="s">
-        <v>439</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>440</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="30"/>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="31" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="31" t="s">
-        <v>444</v>
+      <c r="I36" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11">
+      <c r="B37" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>